<commit_message>
fix endpoint ordenes android
</commit_message>
<xml_diff>
--- a/excel/estandares.xlsx
+++ b/excel/estandares.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/899bfed8ee2a0bb2/Documentos/produccion_server_pg/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{BC659E95-4447-4981-B183-C4EBEB171226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB1CF5FC-6D8D-4774-A57B-805AFBA66399}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{BC659E95-4447-4981-B183-C4EBEB171226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE92105E-3F31-4324-80A6-33B044CA247C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{48541B42-76CC-4E9E-B39F-69041010F793}"/>
   </bookViews>
@@ -456,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C42F5BF-A3CF-4E97-9468-70008ABCB2F8}">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -997,966 +997,977 @@
         <v>48</v>
       </c>
       <c r="B49" s="2">
-        <v>9.3872229465449735</v>
+        <v>3</v>
       </c>
       <c r="C49" s="4">
-        <v>1880.1047499451047</v>
+        <v>5850</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" s="2">
-        <v>2.7554535017221582</v>
+        <v>9.3872229465449735</v>
       </c>
       <c r="C50" s="4">
-        <v>6405.1026226943359</v>
+        <v>1880.1047499451047</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="2">
-        <v>4.234297812279463</v>
+        <v>2.7554535017221582</v>
       </c>
       <c r="C51" s="4">
-        <v>4168.0966320816869</v>
+        <v>6405.1026226943359</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" s="2">
-        <v>1.8461538461538463</v>
+        <v>4.234297812279463</v>
       </c>
       <c r="C52" s="4">
-        <v>9559.8546607378139</v>
+        <v>4168.0966320816869</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B53" s="2">
-        <v>2.7831465017394721</v>
+        <v>1.8461538461538463</v>
       </c>
       <c r="C53" s="4">
-        <v>6341.3702582894039</v>
+        <v>9559.8546607378139</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" s="2">
-        <v>5.7097541633624127</v>
+        <v>2.7831465017394721</v>
       </c>
       <c r="C54" s="4">
-        <v>3091.0196736385587</v>
+        <v>6341.3702582894039</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="2">
-        <v>3.7676609105180532</v>
+        <v>5.7097541633624127</v>
       </c>
       <c r="C55" s="4">
-        <v>4684.3287837615289</v>
+        <v>3091.0196736385587</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" s="2">
-        <v>3.9560439560439447</v>
+        <v>3.7676609105180532</v>
       </c>
       <c r="C56" s="4">
-        <v>4461.265508344326</v>
+        <v>4684.3287837615289</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" s="2">
-        <v>8.3916083916083917</v>
+        <v>3.9560439560439447</v>
       </c>
       <c r="C57" s="4">
-        <v>2103.168025362319</v>
+        <v>4461.265508344326</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" s="2">
-        <v>3.397829164700338</v>
+        <v>8.3916083916083917</v>
       </c>
       <c r="C58" s="4">
-        <v>5194.1876990008668</v>
+        <v>2103.168025362319</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" s="2">
-        <v>5.3771471247199418</v>
+        <v>3.397829164700338</v>
       </c>
       <c r="C59" s="4">
-        <v>3282.2167668533152</v>
+        <v>5194.1876990008668</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B60" s="2">
-        <v>1.5915119363395225</v>
+        <v>5.3771471247199418</v>
       </c>
       <c r="C60" s="4">
-        <v>11089.431406455866</v>
+        <v>3282.2167668533152</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B61" s="2">
-        <v>0.66889632107023411</v>
+        <v>1.5915119363395225</v>
       </c>
       <c r="C61" s="4">
-        <v>26385.198863636368</v>
+        <v>11089.431406455866</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B62" s="2">
-        <v>4.858299595141701</v>
+        <v>0.66889632107023411</v>
       </c>
       <c r="C62" s="4">
-        <v>3632.744771080369</v>
+        <v>26385.198863636368</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B63" s="2">
-        <v>3.0769230769230771</v>
+        <v>4.858299595141701</v>
       </c>
       <c r="C63" s="4">
-        <v>5735.912796442688</v>
+        <v>3632.744771080369</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B64" s="2">
-        <v>0.12474012474012475</v>
+        <v>3.0769230769230771</v>
       </c>
       <c r="C64" s="4">
-        <v>141485.84897891965</v>
+        <v>5735.912796442688</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="2">
-        <v>2.4</v>
+        <v>0.12474012474012475</v>
       </c>
       <c r="C65" s="4">
-        <v>7265.489542160738</v>
+        <v>141485.84897891965</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B66" s="2">
-        <v>5.1858254105445116</v>
+        <v>2.4</v>
       </c>
       <c r="C66" s="4">
-        <v>3403.3082592226619</v>
+        <v>7265.489542160738</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B67" s="2">
-        <v>5.7692307692307692</v>
+        <v>5.1858254105445116</v>
       </c>
       <c r="C67" s="4">
-        <v>3059.1534914361005</v>
+        <v>3403.3082592226619</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B68" s="2">
-        <v>4.7581284694686756</v>
+        <v>5.7692307692307692</v>
       </c>
       <c r="C68" s="4">
-        <v>3709.2236083662715</v>
+        <v>3059.1534914361005</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B69" s="2">
-        <v>5.1282051282051277</v>
+        <v>4.7581284694686756</v>
       </c>
       <c r="C69" s="4">
-        <v>3441.5476778656134</v>
+        <v>3709.2236083662715</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B70" s="2">
-        <v>6.3224446786090622</v>
+        <v>5.1282051282051277</v>
       </c>
       <c r="C70" s="4">
-        <v>2791.4775609354419</v>
+        <v>3441.5476778656134</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B71" s="2">
-        <v>3.5502958579881652</v>
+        <v>6.3224446786090622</v>
       </c>
       <c r="C71" s="4">
-        <v>4971.1244235836639</v>
+        <v>2791.4775609354419</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B72" s="2">
-        <v>8.7082728592162564</v>
+        <v>3.5502958579881652</v>
       </c>
       <c r="C72" s="4">
-        <v>2026.6891880764165</v>
+        <v>4971.1244235836639</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B73" s="2">
-        <v>5.4945054945054936</v>
+        <v>8.7082728592162564</v>
       </c>
       <c r="C73" s="4">
-        <v>3212.1111660079059</v>
+        <v>2026.6891880764165</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B74" s="2">
-        <v>7.1005917159763303</v>
+        <v>5.4945054945054936</v>
       </c>
       <c r="C74" s="4">
-        <v>2485.5622117918319</v>
+        <v>3212.1111660079059</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B75" s="2">
-        <v>4.615384615384615</v>
+        <v>7.1005917159763303</v>
       </c>
       <c r="C75" s="4">
-        <v>3823.9418642951255</v>
+        <v>2485.5622117918319</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B76" s="2">
-        <v>1.1538461538461537</v>
+        <v>4.615384615384615</v>
       </c>
       <c r="C76" s="4">
-        <v>15295.767457180502</v>
+        <v>3823.9418642951255</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B77" s="2">
-        <v>1.3186813186813187</v>
+        <v>1.1538461538461537</v>
       </c>
       <c r="C77" s="4">
-        <v>13383.79652503294</v>
+        <v>15295.767457180502</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B78" s="2">
-        <v>1.741654571843251</v>
+        <v>1.3186813186813187</v>
       </c>
       <c r="C78" s="4">
-        <v>10133.445940382084</v>
+        <v>13383.79652503294</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B79" s="2">
-        <v>2.5641025641025639</v>
+        <v>1.741654571843251</v>
       </c>
       <c r="C79" s="4">
-        <v>6883.0953557312268</v>
+        <v>10133.445940382084</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B80" s="2">
-        <v>1.1732040201791092</v>
+        <v>2.5641025641025639</v>
       </c>
       <c r="C80" s="4">
-        <v>15043.387294137025</v>
+        <v>6883.0953557312268</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B81" s="2">
-        <v>2.4</v>
+        <v>1.1732040201791092</v>
       </c>
       <c r="C81" s="4">
-        <v>7265.489542160738</v>
+        <v>15043.387294137025</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B82" s="2">
-        <v>2.3076923076923075</v>
+        <v>2.4</v>
       </c>
       <c r="C82" s="4">
-        <v>7647.8837285902509</v>
+        <v>7265.489542160738</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B83" s="2">
-        <v>3.6923076923076925</v>
+        <v>2.3076923076923075</v>
       </c>
       <c r="C83" s="4">
-        <v>4779.927330368907</v>
+        <v>7647.8837285902509</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B84" s="2">
-        <v>3.8461538461538458</v>
+        <v>3.6923076923076925</v>
       </c>
       <c r="C84" s="4">
-        <v>4588.7302371541509</v>
+        <v>4779.927330368907</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B85" s="2">
-        <v>2.8846153846153846</v>
+        <v>3.8461538461538458</v>
       </c>
       <c r="C85" s="4">
-        <v>6118.3069828722009</v>
+        <v>4588.7302371541509</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B86" s="2">
-        <v>3.183023872679045</v>
+        <v>2.8846153846153846</v>
       </c>
       <c r="C86" s="4">
-        <v>5544.7157032279329</v>
+        <v>6118.3069828722009</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B87" s="2">
-        <v>5.7692307692307692</v>
+        <v>3.183023872679045</v>
       </c>
       <c r="C87" s="4">
-        <v>3059.1534914361005</v>
+        <v>5544.7157032279329</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B88" s="2">
-        <v>2.5359256128486898</v>
+        <v>5.7692307692307692</v>
       </c>
       <c r="C88" s="4">
-        <v>6959.5741930171289</v>
+        <v>3059.1534914361005</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B89" s="2">
-        <v>4.1580041580041582</v>
+        <v>2.5359256128486898</v>
       </c>
       <c r="C89" s="4">
-        <v>4244.575469367589</v>
+        <v>6959.5741930171289</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B90" s="2">
-        <v>5.4945054945054936</v>
+        <v>4.1580041580041582</v>
       </c>
       <c r="C90" s="4">
-        <v>3212.1111660079059</v>
+        <v>4244.575469367589</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B91" s="2">
-        <v>9.615384615384615</v>
+        <v>5.4945054945054936</v>
       </c>
       <c r="C91" s="4">
-        <v>1835.4920948616602</v>
+        <v>3212.1111660079059</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B92" s="2">
-        <v>2.1978021978021975</v>
+        <v>9.615384615384615</v>
       </c>
       <c r="C92" s="4">
-        <v>8030.2779150197639</v>
+        <v>1835.4920948616602</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B93" s="2">
-        <v>6.593406593406594</v>
+        <v>2.1978021978021975</v>
       </c>
       <c r="C93" s="4">
-        <v>2676.759305006588</v>
+        <v>8030.2779150197639</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B94" s="2">
-        <v>1.5412829425146417</v>
-      </c>
-      <c r="C94" s="5">
-        <v>11450.825778813954</v>
+        <v>6.593406593406594</v>
+      </c>
+      <c r="C94" s="4">
+        <v>2676.759305006588</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B95" s="2">
-        <v>2.0901432328709855</v>
+        <v>1.5412829425146417</v>
       </c>
       <c r="C95" s="5">
-        <v>8443.9009600076879</v>
+        <v>11450.825778813954</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B96" s="2">
-        <v>2.4</v>
-      </c>
-      <c r="C96" s="4">
-        <v>7265.489542160738</v>
+        <v>2.0901432328709855</v>
+      </c>
+      <c r="C96" s="5">
+        <v>8443.9009600076879</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B97" s="2">
-        <v>1.0077258985555928</v>
-      </c>
-      <c r="C97" s="5">
-        <v>17513.653738471676</v>
+        <v>2.4</v>
+      </c>
+      <c r="C97" s="4">
+        <v>7265.489542160738</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B98" s="2">
-        <v>2.3076923076923075</v>
+        <v>1.0077258985555928</v>
       </c>
       <c r="C98" s="5">
-        <v>7647.8837285902509</v>
+        <v>17513.653738471676</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B99" s="2">
-        <v>0.50167224080267558</v>
+        <v>2.3076923076923075</v>
       </c>
       <c r="C99" s="5">
-        <v>35180.265151515159</v>
+        <v>7647.8837285902509</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B100" s="2">
-        <v>2.1567217828900072</v>
+        <v>0.50167224080267558</v>
       </c>
       <c r="C100" s="5">
-        <v>8183.2355895915689</v>
+        <v>35180.265151515159</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B101" s="2">
-        <v>2.5289778714436246</v>
+        <v>2.1567217828900072</v>
       </c>
       <c r="C101" s="5">
-        <v>6978.6939023386049</v>
+        <v>8183.2355895915689</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B102" s="2">
-        <v>3.8461538461538458</v>
+        <v>2.5289778714436246</v>
       </c>
       <c r="C102" s="5">
-        <v>4588.7302371541509</v>
+        <v>6978.6939023386049</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B103" s="2">
-        <v>3.296703296703297</v>
+        <v>3.8461538461538458</v>
       </c>
       <c r="C103" s="5">
-        <v>5353.5186100131759</v>
+        <v>4588.7302371541509</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B104" s="2">
-        <v>3.6427660737053</v>
+        <v>3.296703296703297</v>
       </c>
       <c r="C104" s="5">
-        <v>4844.9343420619243</v>
+        <v>5353.5186100131759</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B105" s="2">
-        <v>8.1400081400081401</v>
+        <v>3.6427660737053</v>
       </c>
       <c r="C105" s="5">
-        <v>2168.1750370553364</v>
+        <v>4844.9343420619243</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B106" s="2">
-        <v>0</v>
-      </c>
-      <c r="C106" s="4">
-        <v>0</v>
+        <v>8.1400081400081401</v>
+      </c>
+      <c r="C106" s="5">
+        <v>2168.1750370553364</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B107" s="2">
-        <v>0.65934065934065933</v>
-      </c>
-      <c r="C107" s="5">
-        <v>26767.59305006588</v>
+        <v>0</v>
+      </c>
+      <c r="C107" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B108" s="2">
-        <v>6.3224446786090622</v>
+        <v>0.65934065934065933</v>
       </c>
       <c r="C108" s="5">
-        <v>2791.4775609354419</v>
+        <v>26767.59305006588</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B109" s="2">
-        <v>0.44911639605170695</v>
+        <v>6.3224446786090622</v>
       </c>
       <c r="C109" s="5">
-        <v>39297.078899254782</v>
+        <v>2791.4775609354419</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B110" s="2">
-        <v>1.1259781935556514</v>
+        <v>0.44911639605170695</v>
       </c>
       <c r="C110" s="5">
-        <v>15674.337701745722</v>
+        <v>39297.078899254782</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B111" s="2">
-        <v>2.4</v>
-      </c>
-      <c r="C111" s="4">
-        <v>7265.489542160738</v>
+        <v>1.1259781935556514</v>
+      </c>
+      <c r="C111" s="5">
+        <v>15674.337701745722</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B112" s="2">
-        <v>1.0077258985555928</v>
-      </c>
-      <c r="C112" s="5">
-        <v>17513.653738471676</v>
+        <v>2.4</v>
+      </c>
+      <c r="C112" s="4">
+        <v>7265.489542160738</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B113" s="2">
-        <v>2.3076923076923075</v>
+        <v>1.0077258985555928</v>
       </c>
       <c r="C113" s="5">
-        <v>7647.8837285902509</v>
+        <v>17513.653738471676</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B114" s="2">
-        <v>0.41958041958041958</v>
+        <v>2.3076923076923075</v>
       </c>
       <c r="C114" s="5">
-        <v>42063.360507246383</v>
+        <v>7647.8837285902509</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B115" s="2">
-        <v>2.1567217828900072</v>
+        <v>0.41958041958041958</v>
       </c>
       <c r="C115" s="5">
-        <v>8183.2355895915689</v>
+        <v>42063.360507246383</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B116" s="2">
-        <v>2.5289778714436246</v>
+        <v>2.1567217828900072</v>
       </c>
       <c r="C116" s="5">
-        <v>6978.6939023386049</v>
+        <v>8183.2355895915689</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B117" s="2">
-        <v>3.8461538461538458</v>
+        <v>2.5289778714436246</v>
       </c>
       <c r="C117" s="5">
-        <v>4588.7302371541509</v>
+        <v>6978.6939023386049</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B118" s="2">
-        <v>3.296703296703297</v>
+        <v>3.8461538461538458</v>
       </c>
       <c r="C118" s="5">
-        <v>5353.5186100131759</v>
+        <v>4588.7302371541509</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B119" s="2">
-        <v>3.6427660737053</v>
+        <v>3.296703296703297</v>
       </c>
       <c r="C119" s="5">
-        <v>4844.9343420619243</v>
+        <v>5353.5186100131759</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B120" s="2">
-        <v>8.1400081400081401</v>
+        <v>3.6427660737053</v>
       </c>
       <c r="C120" s="5">
-        <v>2168.1750370553364</v>
+        <v>4844.9343420619243</v>
       </c>
     </row>
     <row r="121" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B121" s="2">
-        <v>13.186813186813188</v>
+        <v>8.1400081400081401</v>
       </c>
       <c r="C121" s="5">
-        <v>1338.379652503294</v>
+        <v>2168.1750370553364</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B122" s="2">
-        <v>12.474012474012472</v>
+        <v>13.186813186813188</v>
       </c>
       <c r="C122" s="5">
-        <v>1414.8584897891967</v>
+        <v>1338.379652503294</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B123" s="2">
-        <v>10.733452593917711</v>
+        <v>12.474012474012472</v>
       </c>
       <c r="C123" s="5">
-        <v>1644.295001646904</v>
+        <v>1414.8584897891967</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B124" s="2">
-        <v>4.1958041958041958</v>
+        <v>10.733452593917711</v>
       </c>
       <c r="C124" s="5">
-        <v>4206.336050724638</v>
+        <v>1644.295001646904</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B125" s="2">
-        <v>7.1556350626118066</v>
+        <v>4.1958041958041958</v>
       </c>
       <c r="C125" s="5">
-        <v>2466.442502470356</v>
+        <v>4206.336050724638</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B126" s="2">
-        <v>7.9166116901965955</v>
+        <v>7.1556350626118066</v>
       </c>
       <c r="C126" s="5">
-        <v>2229.3581068840585</v>
+        <v>2466.442502470356</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B127" s="2">
-        <v>27.63703362505758</v>
+        <v>7.9166116901965955</v>
       </c>
       <c r="C127" s="5">
-        <v>638.5982913372859</v>
+        <v>2229.3581068840585</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B128" s="2">
-        <v>14.201183431952661</v>
+        <v>27.63703362505758</v>
       </c>
       <c r="C128" s="5">
-        <v>1242.781105895916</v>
+        <v>638.5982913372859</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B129" s="2">
-        <v>9.883050568275408</v>
+        <v>14.201183431952661</v>
       </c>
       <c r="C129" s="5">
-        <v>1785.7808506258236</v>
+        <v>1242.781105895916</v>
       </c>
     </row>
     <row r="130" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B130" s="2">
-        <v>0.8708272859216255</v>
+        <v>9.883050568275408</v>
       </c>
       <c r="C130" s="5">
-        <v>20266.891880764168</v>
+        <v>1785.7808506258236</v>
       </c>
     </row>
     <row r="131" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B131" s="2">
-        <v>1.3986013986013985</v>
+        <v>0.8708272859216255</v>
       </c>
       <c r="C131" s="5">
-        <v>12619.008152173914</v>
+        <v>20266.891880764168</v>
       </c>
     </row>
     <row r="132" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="3">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B132" s="2">
-        <v>0.42735042735042733</v>
+        <v>1.3986013986013985</v>
       </c>
       <c r="C132" s="5">
-        <v>41298.572134387359</v>
+        <v>12619.008152173914</v>
       </c>
     </row>
     <row r="133" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="3">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B133" s="2">
-        <v>6.3224446786090622</v>
+        <v>0.42735042735042733</v>
       </c>
       <c r="C133" s="5">
-        <v>2791.4775609354419</v>
+        <v>41298.572134387359</v>
       </c>
     </row>
     <row r="134" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="3">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B134" s="2">
-        <v>0.25</v>
+        <v>6.3224446786090622</v>
       </c>
       <c r="C134" s="5">
-        <v>70595.849802371551</v>
+        <v>2791.4775609354419</v>
       </c>
     </row>
     <row r="135" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B135" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.25</v>
       </c>
       <c r="C135" s="5">
-        <v>26473.443675889332</v>
+        <v>70595.849802371551</v>
       </c>
     </row>
     <row r="136" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
+        <v>134</v>
+      </c>
+      <c r="B136" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C136" s="5">
+        <v>26473.443675889332</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A137" s="3">
         <v>135</v>
       </c>
-      <c r="B136" s="2">
+      <c r="B137" s="2">
         <v>1</v>
       </c>
-      <c r="C136" s="5">
+      <c r="C137" s="5">
         <v>17648.962450592888</v>
       </c>
     </row>

</xml_diff>